<commit_message>
Update FY27 Education Classes Roster.xlsx
</commit_message>
<xml_diff>
--- a/training/upload/FY27 Education Classes Roster.xlsx
+++ b/training/upload/FY27 Education Classes Roster.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aaronbell/Desktop/Git Repo Clone/CrewOps360/training/upload/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5a8cad284f0e3288/Desktop/GitHub Repo/CrewOps360/training/upload/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F110773-D84F-C44C-B85F-5CAEF7030B1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{0F110773-D84F-C44C-B85F-5CAEF7030B1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B193B240-2E47-49C8-8139-2F8B4A24D9C5}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17260" activeTab="6" xr2:uid="{5604E27C-0991-9B4E-A9D1-5F87A876A78F}"/>
+    <workbookView xWindow="1395" yWindow="945" windowWidth="22995" windowHeight="13260" xr2:uid="{5604E27C-0991-9B4E-A9D1-5F87A876A78F}"/>
   </bookViews>
   <sheets>
     <sheet name="Class_Enrollment" sheetId="1" r:id="rId1"/>
@@ -1180,20 +1180,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AE3E758-B252-634C-B9B3-AE34AE7DE6C7}">
   <dimension ref="A1:K151"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.83203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" style="1" customWidth="1"/>
-    <col min="5" max="6" width="16.6640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="19.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.875" style="1" customWidth="1"/>
+    <col min="5" max="6" width="16.625" style="1" customWidth="1"/>
     <col min="7" max="7" width="22" style="1" customWidth="1"/>
-    <col min="8" max="8" width="20.1640625" style="1" customWidth="1"/>
-    <col min="9" max="11" width="16.6640625" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="10.83203125" style="1"/>
+    <col min="8" max="8" width="20.125" style="1" customWidth="1"/>
+    <col min="9" max="11" width="16.625" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="10.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1228,7 +1228,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -1260,7 +1260,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
@@ -1295,7 +1295,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -1327,7 +1327,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -1359,7 +1359,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
@@ -1391,7 +1391,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
@@ -1426,7 +1426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>18</v>
       </c>
@@ -1461,7 +1461,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>19</v>
       </c>
@@ -1493,7 +1493,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>20</v>
       </c>
@@ -1525,7 +1525,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>21</v>
       </c>
@@ -1557,7 +1557,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
@@ -1589,7 +1589,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>23</v>
       </c>
@@ -1621,7 +1621,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
@@ -1653,7 +1653,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>25</v>
       </c>
@@ -1685,7 +1685,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>26</v>
       </c>
@@ -1717,7 +1717,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>27</v>
       </c>
@@ -1749,7 +1749,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>28</v>
       </c>
@@ -1781,7 +1781,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>29</v>
       </c>
@@ -1813,7 +1813,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>30</v>
       </c>
@@ -1845,7 +1845,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>31</v>
       </c>
@@ -1877,7 +1877,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>32</v>
       </c>
@@ -1909,7 +1909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>33</v>
       </c>
@@ -1941,7 +1941,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>34</v>
       </c>
@@ -1973,7 +1973,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>35</v>
       </c>
@@ -2005,7 +2005,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>36</v>
       </c>
@@ -2037,7 +2037,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>37</v>
       </c>
@@ -2069,7 +2069,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>38</v>
       </c>
@@ -2104,7 +2104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>39</v>
       </c>
@@ -2136,7 +2136,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>40</v>
       </c>
@@ -2168,7 +2168,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>41</v>
       </c>
@@ -2200,7 +2200,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>42</v>
       </c>
@@ -2232,7 +2232,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>43</v>
       </c>
@@ -2264,7 +2264,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>44</v>
       </c>
@@ -2296,7 +2296,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>45</v>
       </c>
@@ -2328,7 +2328,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>46</v>
       </c>
@@ -2360,7 +2360,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>47</v>
       </c>
@@ -2392,7 +2392,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>48</v>
       </c>
@@ -2424,7 +2424,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>49</v>
       </c>
@@ -2459,7 +2459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>50</v>
       </c>
@@ -2491,7 +2491,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>51</v>
       </c>
@@ -2523,7 +2523,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>52</v>
       </c>
@@ -2558,7 +2558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>53</v>
       </c>
@@ -2590,7 +2590,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>54</v>
       </c>
@@ -2622,7 +2622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>55</v>
       </c>
@@ -2657,7 +2657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>57</v>
       </c>
@@ -2689,7 +2689,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>58</v>
       </c>
@@ -2721,7 +2721,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>59</v>
       </c>
@@ -2753,7 +2753,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>60</v>
       </c>
@@ -2785,7 +2785,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>61</v>
       </c>
@@ -2817,7 +2817,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>62</v>
       </c>
@@ -2849,7 +2849,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>63</v>
       </c>
@@ -2881,7 +2881,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>64</v>
       </c>
@@ -2916,7 +2916,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>65</v>
       </c>
@@ -2951,7 +2951,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>66</v>
       </c>
@@ -2983,7 +2983,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>67</v>
       </c>
@@ -3018,7 +3018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>68</v>
       </c>
@@ -3053,7 +3053,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>69</v>
       </c>
@@ -3085,7 +3085,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>70</v>
       </c>
@@ -3117,7 +3117,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>71</v>
       </c>
@@ -3149,7 +3149,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>72</v>
       </c>
@@ -3181,7 +3181,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>73</v>
       </c>
@@ -3216,7 +3216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>74</v>
       </c>
@@ -3248,7 +3248,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>75</v>
       </c>
@@ -3265,7 +3265,7 @@
         <v>0</v>
       </c>
       <c r="F64" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G64" s="2" t="b">
         <v>1</v>
@@ -3283,7 +3283,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>76</v>
       </c>
@@ -3315,7 +3315,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>77</v>
       </c>
@@ -3347,7 +3347,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>78</v>
       </c>
@@ -3379,7 +3379,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>79</v>
       </c>
@@ -3411,7 +3411,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>80</v>
       </c>
@@ -3443,7 +3443,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>81</v>
       </c>
@@ -3475,7 +3475,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>82</v>
       </c>
@@ -3510,7 +3510,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>83</v>
       </c>
@@ -3542,7 +3542,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>84</v>
       </c>
@@ -3574,7 +3574,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>85</v>
       </c>
@@ -3606,7 +3606,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>86</v>
       </c>
@@ -3638,7 +3638,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>87</v>
       </c>
@@ -3670,7 +3670,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>88</v>
       </c>
@@ -3705,7 +3705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>89</v>
       </c>
@@ -3737,7 +3737,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>90</v>
       </c>
@@ -3769,7 +3769,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>91</v>
       </c>
@@ -3801,7 +3801,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>92</v>
       </c>
@@ -3833,7 +3833,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>93</v>
       </c>
@@ -3865,7 +3865,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>94</v>
       </c>
@@ -3897,7 +3897,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>95</v>
       </c>
@@ -3929,7 +3929,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>96</v>
       </c>
@@ -3958,7 +3958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>97</v>
       </c>
@@ -3969,7 +3969,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>99</v>
       </c>
@@ -3980,7 +3980,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>100</v>
       </c>
@@ -3991,7 +3991,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>101</v>
       </c>
@@ -4002,7 +4002,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>102</v>
       </c>
@@ -4013,7 +4013,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>103</v>
       </c>
@@ -4042,7 +4042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>104</v>
       </c>
@@ -4053,7 +4053,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>105</v>
       </c>
@@ -4064,7 +4064,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>106</v>
       </c>
@@ -4075,7 +4075,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>107</v>
       </c>
@@ -4086,7 +4086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>108</v>
       </c>
@@ -4097,7 +4097,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>109</v>
       </c>
@@ -4108,7 +4108,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>110</v>
       </c>
@@ -4119,7 +4119,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>111</v>
       </c>
@@ -4130,7 +4130,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>112</v>
       </c>
@@ -4141,7 +4141,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>113</v>
       </c>
@@ -4152,7 +4152,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>114</v>
       </c>
@@ -4163,7 +4163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>116</v>
       </c>
@@ -4174,7 +4174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>117</v>
       </c>
@@ -4185,7 +4185,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>118</v>
       </c>
@@ -4196,7 +4196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>119</v>
       </c>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>120</v>
       </c>
@@ -4218,7 +4218,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>121</v>
       </c>
@@ -4229,7 +4229,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>122</v>
       </c>
@@ -4240,7 +4240,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>123</v>
       </c>
@@ -4251,7 +4251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>124</v>
       </c>
@@ -4262,7 +4262,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>125</v>
       </c>
@@ -4273,7 +4273,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>126</v>
       </c>
@@ -4284,7 +4284,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>127</v>
       </c>
@@ -4295,7 +4295,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>128</v>
       </c>
@@ -4306,7 +4306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>129</v>
       </c>
@@ -4317,7 +4317,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>110</v>
       </c>
@@ -4328,7 +4328,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
         <v>130</v>
       </c>
@@ -4339,7 +4339,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>131</v>
       </c>
@@ -4350,7 +4350,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>132</v>
       </c>
@@ -4361,7 +4361,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>133</v>
       </c>
@@ -4372,7 +4372,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
         <v>134</v>
       </c>
@@ -4383,7 +4383,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>136</v>
       </c>
@@ -4394,7 +4394,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>137</v>
       </c>
@@ -4405,7 +4405,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>138</v>
       </c>
@@ -4416,7 +4416,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>139</v>
       </c>
@@ -4427,7 +4427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>140</v>
       </c>
@@ -4438,7 +4438,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
         <v>141</v>
       </c>
@@ -4449,7 +4449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>142</v>
       </c>
@@ -4460,7 +4460,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
         <v>143</v>
       </c>
@@ -4471,7 +4471,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
         <v>144</v>
       </c>
@@ -4482,7 +4482,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
         <v>145</v>
       </c>
@@ -4493,7 +4493,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
         <v>147</v>
       </c>
@@ -4504,7 +4504,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
         <v>148</v>
       </c>
@@ -4515,7 +4515,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
         <v>149</v>
       </c>
@@ -4526,7 +4526,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
         <v>150</v>
       </c>
@@ -4537,7 +4537,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
         <v>151</v>
       </c>
@@ -4548,7 +4548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
         <v>152</v>
       </c>
@@ -4559,7 +4559,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
         <v>153</v>
       </c>
@@ -4570,7 +4570,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
         <v>154</v>
       </c>
@@ -4581,7 +4581,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
         <v>155</v>
       </c>
@@ -4592,7 +4592,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
         <v>156</v>
       </c>
@@ -4603,7 +4603,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
         <v>157</v>
       </c>
@@ -4614,7 +4614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
         <v>158</v>
       </c>
@@ -4625,7 +4625,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
         <v>159</v>
       </c>
@@ -4636,7 +4636,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>160</v>
       </c>
@@ -4647,7 +4647,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
         <v>161</v>
       </c>
@@ -4658,7 +4658,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
         <v>162</v>
       </c>
@@ -4669,10 +4669,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F151" s="1">
         <f>COUNTIF(Table2[CRM],TRUE)</f>
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -4686,21 +4686,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C57329F-C782-4ACF-89E8-E29E38627636}">
   <dimension ref="A1:I28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="10.83203125" style="1"/>
+    <col min="8" max="8" width="15.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="10.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>163</v>
       </c>
@@ -4726,7 +4726,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>167</v>
       </c>
@@ -4749,7 +4749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>168</v>
       </c>
@@ -4763,7 +4763,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>169</v>
       </c>
@@ -4775,7 +4775,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>170</v>
       </c>
@@ -4787,7 +4787,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>171</v>
       </c>
@@ -4799,7 +4799,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>172</v>
       </c>
@@ -4811,7 +4811,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>173</v>
       </c>
@@ -4823,7 +4823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>174</v>
       </c>
@@ -4835,7 +4835,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>175</v>
       </c>
@@ -4847,7 +4847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>176</v>
       </c>
@@ -4859,7 +4859,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>177</v>
       </c>
@@ -4871,7 +4871,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>178</v>
       </c>
@@ -4883,7 +4883,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>179</v>
       </c>
@@ -4895,7 +4895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C15" s="6" t="s">
         <v>180</v>
       </c>
@@ -4906,7 +4906,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>183</v>
       </c>
@@ -4914,7 +4914,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>184</v>
       </c>
@@ -4922,7 +4922,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>186</v>
       </c>
@@ -4930,7 +4930,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>187</v>
       </c>
@@ -4938,7 +4938,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>188</v>
       </c>
@@ -4946,7 +4946,7 @@
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>189</v>
       </c>
@@ -4954,41 +4954,41 @@
         <v>0.45833333333333331</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>190</v>
       </c>
       <c r="B22" s="9"/>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>191</v>
       </c>
       <c r="B23" s="9"/>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>192</v>
       </c>
       <c r="B24" s="9"/>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>193</v>
       </c>
       <c r="B25" s="9"/>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>196</v>
       </c>
@@ -5006,21 +5006,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27D6B412-4F13-4653-A9FC-73F2CE560866}">
   <dimension ref="A1:I28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="10.83203125" style="1"/>
+    <col min="8" max="8" width="15.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="10.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>163</v>
       </c>
@@ -5046,7 +5046,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>167</v>
       </c>
@@ -5069,7 +5069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>168</v>
       </c>
@@ -5083,7 +5083,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>169</v>
       </c>
@@ -5095,7 +5095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>170</v>
       </c>
@@ -5107,7 +5107,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>171</v>
       </c>
@@ -5119,7 +5119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>172</v>
       </c>
@@ -5131,7 +5131,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>173</v>
       </c>
@@ -5143,7 +5143,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>174</v>
       </c>
@@ -5155,7 +5155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>175</v>
       </c>
@@ -5167,7 +5167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>176</v>
       </c>
@@ -5179,7 +5179,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>177</v>
       </c>
@@ -5191,7 +5191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>178</v>
       </c>
@@ -5203,7 +5203,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>179</v>
       </c>
@@ -5215,7 +5215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C15" s="6" t="s">
         <v>180</v>
       </c>
@@ -5226,7 +5226,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>183</v>
       </c>
@@ -5234,7 +5234,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>184</v>
       </c>
@@ -5242,7 +5242,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>186</v>
       </c>
@@ -5250,7 +5250,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>187</v>
       </c>
@@ -5258,7 +5258,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>188</v>
       </c>
@@ -5266,7 +5266,7 @@
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>189</v>
       </c>
@@ -5274,41 +5274,41 @@
         <v>0.45833333333333331</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>190</v>
       </c>
       <c r="B22" s="9"/>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>191</v>
       </c>
       <c r="B23" s="9"/>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>192</v>
       </c>
       <c r="B24" s="9"/>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>193</v>
       </c>
       <c r="B25" s="9"/>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>196</v>
       </c>
@@ -5326,20 +5326,20 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88FFB9B6-1164-4865-9A5D-7FFA6B96DA49}">
   <dimension ref="A1:I28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="10.83203125" style="1"/>
+    <col min="8" max="8" width="15.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="10.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>163</v>
       </c>
@@ -5368,7 +5368,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>167</v>
       </c>
@@ -5394,7 +5394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>168</v>
       </c>
@@ -5406,7 +5406,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>169</v>
       </c>
@@ -5418,7 +5418,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>170</v>
       </c>
@@ -5430,7 +5430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>171</v>
       </c>
@@ -5442,7 +5442,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>172</v>
       </c>
@@ -5454,7 +5454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>173</v>
       </c>
@@ -5466,7 +5466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>174</v>
       </c>
@@ -5478,7 +5478,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>175</v>
       </c>
@@ -5490,7 +5490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>176</v>
       </c>
@@ -5502,7 +5502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>177</v>
       </c>
@@ -5514,7 +5514,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>178</v>
       </c>
@@ -5526,7 +5526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>179</v>
       </c>
@@ -5538,7 +5538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C15" s="6" t="s">
         <v>180</v>
       </c>
@@ -5549,7 +5549,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>183</v>
       </c>
@@ -5557,7 +5557,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>184</v>
       </c>
@@ -5565,7 +5565,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>186</v>
       </c>
@@ -5573,7 +5573,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>187</v>
       </c>
@@ -5581,7 +5581,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>188</v>
       </c>
@@ -5589,7 +5589,7 @@
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>189</v>
       </c>
@@ -5597,41 +5597,41 @@
         <v>0.66666666666666663</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>190</v>
       </c>
       <c r="B22" s="9"/>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>191</v>
       </c>
       <c r="B23" s="9"/>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>192</v>
       </c>
       <c r="B24" s="9"/>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>193</v>
       </c>
       <c r="B25" s="9"/>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>196</v>
       </c>
@@ -5652,20 +5652,20 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30857C8E-EA32-4055-B3FC-BF21867CAA9C}">
   <dimension ref="A1:I28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="10.83203125" style="1"/>
+    <col min="8" max="8" width="15.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="10.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>163</v>
       </c>
@@ -5694,7 +5694,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>167</v>
       </c>
@@ -5720,7 +5720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>168</v>
       </c>
@@ -5737,7 +5737,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>169</v>
       </c>
@@ -5754,7 +5754,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>170</v>
       </c>
@@ -5771,7 +5771,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>171</v>
       </c>
@@ -5788,7 +5788,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>172</v>
       </c>
@@ -5805,7 +5805,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>173</v>
       </c>
@@ -5822,7 +5822,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>174</v>
       </c>
@@ -5839,7 +5839,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>175</v>
       </c>
@@ -5851,7 +5851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>176</v>
       </c>
@@ -5863,7 +5863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>177</v>
       </c>
@@ -5875,7 +5875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>178</v>
       </c>
@@ -5887,7 +5887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>179</v>
       </c>
@@ -5899,7 +5899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C15" s="6" t="s">
         <v>180</v>
       </c>
@@ -5910,7 +5910,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>183</v>
       </c>
@@ -5918,7 +5918,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>184</v>
       </c>
@@ -5926,7 +5926,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>186</v>
       </c>
@@ -5934,7 +5934,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>187</v>
       </c>
@@ -5942,7 +5942,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>188</v>
       </c>
@@ -5950,7 +5950,7 @@
         <v>0.41666666666666669</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>189</v>
       </c>
@@ -5958,7 +5958,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>190</v>
       </c>
@@ -5966,7 +5966,7 @@
         <v>0.54166666666666663</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>191</v>
       </c>
@@ -5974,29 +5974,29 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>192</v>
       </c>
       <c r="B24" s="9"/>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>193</v>
       </c>
       <c r="B25" s="9"/>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>196</v>
       </c>
@@ -6017,20 +6017,20 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3179E733-F1FB-41C8-B555-77774997D9E6}">
   <dimension ref="A1:I28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="10.83203125" style="1"/>
+    <col min="8" max="8" width="15.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="10.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>163</v>
       </c>
@@ -6059,7 +6059,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>167</v>
       </c>
@@ -6085,7 +6085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>168</v>
       </c>
@@ -6102,7 +6102,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>169</v>
       </c>
@@ -6119,7 +6119,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>170</v>
       </c>
@@ -6136,7 +6136,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>171</v>
       </c>
@@ -6153,7 +6153,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>172</v>
       </c>
@@ -6170,7 +6170,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>173</v>
       </c>
@@ -6187,7 +6187,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>174</v>
       </c>
@@ -6204,7 +6204,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>175</v>
       </c>
@@ -6221,7 +6221,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>176</v>
       </c>
@@ -6238,7 +6238,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>177</v>
       </c>
@@ -6255,7 +6255,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>178</v>
       </c>
@@ -6267,7 +6267,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>179</v>
       </c>
@@ -6279,7 +6279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C15" s="6" t="s">
         <v>180</v>
       </c>
@@ -6290,7 +6290,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>183</v>
       </c>
@@ -6298,7 +6298,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>184</v>
       </c>
@@ -6306,7 +6306,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>186</v>
       </c>
@@ -6314,7 +6314,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>187</v>
       </c>
@@ -6322,7 +6322,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>188</v>
       </c>
@@ -6330,7 +6330,7 @@
         <v>0.41666666666666669</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>189</v>
       </c>
@@ -6338,7 +6338,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>190</v>
       </c>
@@ -6346,7 +6346,7 @@
         <v>0.54166666666666663</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>191</v>
       </c>
@@ -6354,7 +6354,7 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>192</v>
       </c>
@@ -6362,7 +6362,7 @@
         <v>0.66666666666666663</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>193</v>
       </c>
@@ -6370,17 +6370,17 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>196</v>
       </c>
@@ -6401,21 +6401,21 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCE38F22-476B-47FF-AE37-65825C2770E6}">
   <dimension ref="A1:I28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="10.83203125" style="1"/>
+    <col min="8" max="8" width="15.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="10.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>163</v>
       </c>
@@ -6444,7 +6444,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>167</v>
       </c>
@@ -6470,7 +6470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>168</v>
       </c>
@@ -6487,7 +6487,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>169</v>
       </c>
@@ -6504,7 +6504,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>170</v>
       </c>
@@ -6521,7 +6521,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>171</v>
       </c>
@@ -6533,7 +6533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>172</v>
       </c>
@@ -6545,7 +6545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>173</v>
       </c>
@@ -6557,7 +6557,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>174</v>
       </c>
@@ -6569,7 +6569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>175</v>
       </c>
@@ -6581,7 +6581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>176</v>
       </c>
@@ -6593,7 +6593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>177</v>
       </c>
@@ -6605,7 +6605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>178</v>
       </c>
@@ -6617,7 +6617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>179</v>
       </c>
@@ -6629,7 +6629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C15" s="6" t="s">
         <v>180</v>
       </c>
@@ -6640,7 +6640,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>183</v>
       </c>
@@ -6648,7 +6648,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>184</v>
       </c>
@@ -6656,7 +6656,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>186</v>
       </c>
@@ -6664,7 +6664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>187</v>
       </c>
@@ -6672,7 +6672,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>188</v>
       </c>
@@ -6680,7 +6680,7 @@
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>189</v>
       </c>
@@ -6688,41 +6688,41 @@
         <v>0.66666666666666663</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>190</v>
       </c>
       <c r="B22" s="9"/>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>191</v>
       </c>
       <c r="B23" s="9"/>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>192</v>
       </c>
       <c r="B24" s="9"/>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>193</v>
       </c>
       <c r="B25" s="9"/>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>196</v>
       </c>
@@ -6743,21 +6743,21 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09EEA88E-7AEE-574F-BC90-87FF2ABA87C3}">
   <dimension ref="A1:I28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="10.83203125" style="1"/>
+    <col min="8" max="8" width="15.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="10.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>163</v>
       </c>
@@ -6781,7 +6781,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>167</v>
       </c>
@@ -6802,7 +6802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>168</v>
       </c>
@@ -6814,7 +6814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>169</v>
       </c>
@@ -6826,7 +6826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>170</v>
       </c>
@@ -6838,7 +6838,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>171</v>
       </c>
@@ -6850,7 +6850,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>172</v>
       </c>
@@ -6862,7 +6862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>173</v>
       </c>
@@ -6874,7 +6874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>174</v>
       </c>
@@ -6886,7 +6886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>175</v>
       </c>
@@ -6898,7 +6898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>176</v>
       </c>
@@ -6910,7 +6910,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>177</v>
       </c>
@@ -6922,7 +6922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>178</v>
       </c>
@@ -6934,7 +6934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>179</v>
       </c>
@@ -6946,7 +6946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C15" s="6" t="s">
         <v>180</v>
       </c>
@@ -6957,74 +6957,74 @@
         <v>182</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>186</v>
       </c>
       <c r="B18" s="8"/>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>188</v>
       </c>
       <c r="B20" s="9"/>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>189</v>
       </c>
       <c r="B21" s="9"/>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>190</v>
       </c>
       <c r="B22" s="9"/>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>191</v>
       </c>
       <c r="B23" s="9"/>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>192</v>
       </c>
       <c r="B24" s="9"/>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>193</v>
       </c>
       <c r="B25" s="9"/>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>196</v>
       </c>
@@ -7043,13 +7043,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FE5E83A-B444-4206-8DA8-1368EF05AF5C}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="7" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="7" width="10.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B1" s="3">
         <v>45957</v>
       </c>
@@ -7074,7 +7074,7 @@
         <v>45962</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>97</v>
       </c>
@@ -7097,7 +7097,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>202</v>
       </c>
@@ -7120,7 +7120,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>99</v>
       </c>
@@ -7143,7 +7143,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>100</v>
       </c>
@@ -7166,7 +7166,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>101</v>
       </c>
@@ -7189,7 +7189,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>102</v>
       </c>
@@ -7212,7 +7212,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>204</v>
       </c>
@@ -7235,7 +7235,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>103</v>
       </c>
@@ -7258,7 +7258,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>104</v>
       </c>
@@ -7281,7 +7281,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>105</v>
       </c>
@@ -7304,7 +7304,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>106</v>
       </c>
@@ -7327,7 +7327,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>107</v>
       </c>
@@ -7350,7 +7350,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>108</v>
       </c>
@@ -7373,7 +7373,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>109</v>
       </c>
@@ -7396,7 +7396,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>110</v>
       </c>
@@ -7419,7 +7419,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>111</v>
       </c>
@@ -7442,7 +7442,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>113</v>
       </c>
@@ -7465,7 +7465,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>206</v>
       </c>
@@ -7494,12 +7494,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Flow_SignoffStatus xmlns="3ae64878-e7bb-4c65-a932-4cdc61fbe63f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7686,17 +7685,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Flow_SignoffStatus xmlns="3ae64878-e7bb-4c65-a932-4cdc61fbe63f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBE3643D-FDE0-44DC-9CDA-200C2597DFB6}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13094262-B8A9-472E-A55D-BC65572C19CC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3ae64878-e7bb-4c65-a932-4cdc61fbe63f"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -7721,11 +7723,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13094262-B8A9-472E-A55D-BC65572C19CC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBE3643D-FDE0-44DC-9CDA-200C2597DFB6}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="3ae64878-e7bb-4c65-a932-4cdc61fbe63f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>